<commit_message>
Updating the model for Ulmeni
</commit_message>
<xml_diff>
--- a/Solar Energy Ulmeni/Results_Production_SolarEnergy_xgb.xlsx
+++ b/Solar Energy Ulmeni/Results_Production_SolarEnergy_xgb.xlsx
@@ -28,231 +28,6 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>31.05.202610</t>
-  </si>
-  <si>
-    <t>31.05.202611</t>
-  </si>
-  <si>
-    <t>31.05.202612</t>
-  </si>
-  <si>
-    <t>31.05.202613</t>
-  </si>
-  <si>
-    <t>31.05.202614</t>
-  </si>
-  <si>
-    <t>31.05.202615</t>
-  </si>
-  <si>
-    <t>31.05.202616</t>
-  </si>
-  <si>
-    <t>31.05.202617</t>
-  </si>
-  <si>
-    <t>31.05.202618</t>
-  </si>
-  <si>
-    <t>31.05.202619</t>
-  </si>
-  <si>
-    <t>31.05.202620</t>
-  </si>
-  <si>
-    <t>31.05.202621</t>
-  </si>
-  <si>
-    <t>31.05.202622</t>
-  </si>
-  <si>
-    <t>31.05.202623</t>
-  </si>
-  <si>
-    <t>31.05.202624</t>
-  </si>
-  <si>
-    <t>01.06.20261</t>
-  </si>
-  <si>
-    <t>01.06.20262</t>
-  </si>
-  <si>
-    <t>01.06.20263</t>
-  </si>
-  <si>
-    <t>01.06.20264</t>
-  </si>
-  <si>
-    <t>01.06.20265</t>
-  </si>
-  <si>
-    <t>01.06.20266</t>
-  </si>
-  <si>
-    <t>01.06.20267</t>
-  </si>
-  <si>
-    <t>01.06.20268</t>
-  </si>
-  <si>
-    <t>01.06.20269</t>
-  </si>
-  <si>
-    <t>01.06.202610</t>
-  </si>
-  <si>
-    <t>01.06.202611</t>
-  </si>
-  <si>
-    <t>01.06.202612</t>
-  </si>
-  <si>
-    <t>01.06.202613</t>
-  </si>
-  <si>
-    <t>01.06.202614</t>
-  </si>
-  <si>
-    <t>01.06.202615</t>
-  </si>
-  <si>
-    <t>01.06.202616</t>
-  </si>
-  <si>
-    <t>01.06.202617</t>
-  </si>
-  <si>
-    <t>01.06.202618</t>
-  </si>
-  <si>
-    <t>01.06.202619</t>
-  </si>
-  <si>
-    <t>01.06.202620</t>
-  </si>
-  <si>
-    <t>01.06.202621</t>
-  </si>
-  <si>
-    <t>01.06.202622</t>
-  </si>
-  <si>
-    <t>01.06.202623</t>
-  </si>
-  <si>
-    <t>01.06.202624</t>
-  </si>
-  <si>
-    <t>02.06.20261</t>
-  </si>
-  <si>
-    <t>02.06.20262</t>
-  </si>
-  <si>
-    <t>02.06.20263</t>
-  </si>
-  <si>
-    <t>02.06.20264</t>
-  </si>
-  <si>
-    <t>02.06.20265</t>
-  </si>
-  <si>
-    <t>02.06.20266</t>
-  </si>
-  <si>
-    <t>02.06.20267</t>
-  </si>
-  <si>
-    <t>02.06.20268</t>
-  </si>
-  <si>
-    <t>02.06.20269</t>
-  </si>
-  <si>
-    <t>02.06.202610</t>
-  </si>
-  <si>
-    <t>02.06.202611</t>
-  </si>
-  <si>
-    <t>02.06.202612</t>
-  </si>
-  <si>
-    <t>02.06.202613</t>
-  </si>
-  <si>
-    <t>02.06.202614</t>
-  </si>
-  <si>
-    <t>02.06.202615</t>
-  </si>
-  <si>
-    <t>02.06.202616</t>
-  </si>
-  <si>
-    <t>02.06.202617</t>
-  </si>
-  <si>
-    <t>02.06.202618</t>
-  </si>
-  <si>
-    <t>02.06.202619</t>
-  </si>
-  <si>
-    <t>02.06.202620</t>
-  </si>
-  <si>
-    <t>02.06.202621</t>
-  </si>
-  <si>
-    <t>02.06.202622</t>
-  </si>
-  <si>
-    <t>02.06.202623</t>
-  </si>
-  <si>
-    <t>02.06.202624</t>
-  </si>
-  <si>
-    <t>03.06.20261</t>
-  </si>
-  <si>
-    <t>03.06.20262</t>
-  </si>
-  <si>
-    <t>03.06.20263</t>
-  </si>
-  <si>
-    <t>03.06.20264</t>
-  </si>
-  <si>
-    <t>03.06.20265</t>
-  </si>
-  <si>
-    <t>03.06.20266</t>
-  </si>
-  <si>
-    <t>03.06.20267</t>
-  </si>
-  <si>
-    <t>03.06.20268</t>
-  </si>
-  <si>
-    <t>03.06.20269</t>
-  </si>
-  <si>
-    <t>03.06.202610</t>
-  </si>
-  <si>
-    <t>03.06.202611</t>
-  </si>
-  <si>
-    <t>03.06.202612</t>
-  </si>
-  <si>
     <t>03.06.202613</t>
   </si>
   <si>
@@ -533,6 +308,231 @@
   </si>
   <si>
     <t>07.06.202610</t>
+  </si>
+  <si>
+    <t>07.06.202611</t>
+  </si>
+  <si>
+    <t>07.06.202612</t>
+  </si>
+  <si>
+    <t>07.06.202613</t>
+  </si>
+  <si>
+    <t>07.06.202614</t>
+  </si>
+  <si>
+    <t>07.06.202615</t>
+  </si>
+  <si>
+    <t>07.06.202616</t>
+  </si>
+  <si>
+    <t>07.06.202617</t>
+  </si>
+  <si>
+    <t>07.06.202618</t>
+  </si>
+  <si>
+    <t>07.06.202619</t>
+  </si>
+  <si>
+    <t>07.06.202620</t>
+  </si>
+  <si>
+    <t>07.06.202621</t>
+  </si>
+  <si>
+    <t>07.06.202622</t>
+  </si>
+  <si>
+    <t>07.06.202623</t>
+  </si>
+  <si>
+    <t>07.06.202624</t>
+  </si>
+  <si>
+    <t>08.06.20261</t>
+  </si>
+  <si>
+    <t>08.06.20262</t>
+  </si>
+  <si>
+    <t>08.06.20263</t>
+  </si>
+  <si>
+    <t>08.06.20264</t>
+  </si>
+  <si>
+    <t>08.06.20265</t>
+  </si>
+  <si>
+    <t>08.06.20266</t>
+  </si>
+  <si>
+    <t>08.06.20267</t>
+  </si>
+  <si>
+    <t>08.06.20268</t>
+  </si>
+  <si>
+    <t>08.06.20269</t>
+  </si>
+  <si>
+    <t>08.06.202610</t>
+  </si>
+  <si>
+    <t>08.06.202611</t>
+  </si>
+  <si>
+    <t>08.06.202612</t>
+  </si>
+  <si>
+    <t>08.06.202613</t>
+  </si>
+  <si>
+    <t>08.06.202614</t>
+  </si>
+  <si>
+    <t>08.06.202615</t>
+  </si>
+  <si>
+    <t>08.06.202616</t>
+  </si>
+  <si>
+    <t>08.06.202617</t>
+  </si>
+  <si>
+    <t>08.06.202618</t>
+  </si>
+  <si>
+    <t>08.06.202619</t>
+  </si>
+  <si>
+    <t>08.06.202620</t>
+  </si>
+  <si>
+    <t>08.06.202621</t>
+  </si>
+  <si>
+    <t>08.06.202622</t>
+  </si>
+  <si>
+    <t>08.06.202623</t>
+  </si>
+  <si>
+    <t>08.06.202624</t>
+  </si>
+  <si>
+    <t>09.06.20261</t>
+  </si>
+  <si>
+    <t>09.06.20262</t>
+  </si>
+  <si>
+    <t>09.06.20263</t>
+  </si>
+  <si>
+    <t>09.06.20264</t>
+  </si>
+  <si>
+    <t>09.06.20265</t>
+  </si>
+  <si>
+    <t>09.06.20266</t>
+  </si>
+  <si>
+    <t>09.06.20267</t>
+  </si>
+  <si>
+    <t>09.06.20268</t>
+  </si>
+  <si>
+    <t>09.06.20269</t>
+  </si>
+  <si>
+    <t>09.06.202610</t>
+  </si>
+  <si>
+    <t>09.06.202611</t>
+  </si>
+  <si>
+    <t>09.06.202612</t>
+  </si>
+  <si>
+    <t>09.06.202613</t>
+  </si>
+  <si>
+    <t>09.06.202614</t>
+  </si>
+  <si>
+    <t>09.06.202615</t>
+  </si>
+  <si>
+    <t>09.06.202616</t>
+  </si>
+  <si>
+    <t>09.06.202617</t>
+  </si>
+  <si>
+    <t>09.06.202618</t>
+  </si>
+  <si>
+    <t>09.06.202619</t>
+  </si>
+  <si>
+    <t>09.06.202620</t>
+  </si>
+  <si>
+    <t>09.06.202621</t>
+  </si>
+  <si>
+    <t>09.06.202622</t>
+  </si>
+  <si>
+    <t>09.06.202623</t>
+  </si>
+  <si>
+    <t>09.06.202624</t>
+  </si>
+  <si>
+    <t>10.06.20261</t>
+  </si>
+  <si>
+    <t>10.06.20262</t>
+  </si>
+  <si>
+    <t>10.06.20263</t>
+  </si>
+  <si>
+    <t>10.06.20264</t>
+  </si>
+  <si>
+    <t>10.06.20265</t>
+  </si>
+  <si>
+    <t>10.06.20266</t>
+  </si>
+  <si>
+    <t>10.06.20267</t>
+  </si>
+  <si>
+    <t>10.06.20268</t>
+  </si>
+  <si>
+    <t>10.06.20269</t>
+  </si>
+  <si>
+    <t>10.06.202610</t>
+  </si>
+  <si>
+    <t>10.06.202611</t>
+  </si>
+  <si>
+    <t>10.06.202612</t>
+  </si>
+  <si>
+    <t>10.06.202613</t>
   </si>
 </sst>
 </file>
@@ -913,10 +913,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -927,10 +927,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B3">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B4">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C4">
-        <v>3.481</v>
+        <v>3.509</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B5">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C5">
-        <v>3.384</v>
+        <v>2.955</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C6">
-        <v>3.231</v>
+        <v>2.357</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B7">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C7">
-        <v>3.515</v>
+        <v>1.382</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B8">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C8">
-        <v>2.935</v>
+        <v>0.779</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B9">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C9">
-        <v>2.197</v>
+        <v>0.249</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B10">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C10">
-        <v>0.991</v>
+        <v>0.037</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C11">
-        <v>0.586</v>
+        <v>0</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,13 +1053,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B12">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C12">
-        <v>0.218</v>
+        <v>0</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -1067,13 +1067,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46173</v>
+        <v>46176</v>
       </c>
       <c r="B13">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C13">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B14">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1095,10 +1095,10 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B15">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1109,10 +1109,10 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B16">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1123,10 +1123,10 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1137,10 +1137,10 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -1165,13 +1165,13 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B20">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>0.341</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -1179,13 +1179,13 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B21">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>1.183</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -1193,13 +1193,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B22">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C22">
-        <v>0.028</v>
+        <v>2.169</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B23">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C23">
-        <v>0.334</v>
+        <v>2.798</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B24">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C24">
-        <v>1.07</v>
+        <v>3.05</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B25">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C25">
-        <v>1.831</v>
+        <v>2.98</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B26">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C26">
-        <v>2.644</v>
+        <v>2.743</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B27">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C27">
-        <v>3.33</v>
+        <v>2.649</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B28">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C28">
-        <v>2.601</v>
+        <v>2.269</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B29">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C29">
-        <v>2.012</v>
+        <v>1.75</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B30">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C30">
-        <v>3.462</v>
+        <v>1.176</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B31">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C31">
-        <v>3.283</v>
+        <v>1.034</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B32">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C32">
-        <v>2.46</v>
+        <v>0.478</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B33">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C33">
-        <v>1.554</v>
+        <v>0.148</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B34">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C34">
-        <v>1.056</v>
+        <v>0.014</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B35">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C35">
-        <v>0.505</v>
+        <v>0</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,13 +1389,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B36">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C36">
-        <v>0.173</v>
+        <v>0</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1403,13 +1403,13 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="B37">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C37">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="D37" t="s">
         <v>39</v>
@@ -1417,10 +1417,10 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B38">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1431,10 +1431,10 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B39">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -1445,10 +1445,10 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B40">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -1459,10 +1459,10 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B41">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C41">
         <v>0</v>
@@ -1473,10 +1473,10 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B42">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -1487,13 +1487,13 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B43">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C43">
-        <v>0</v>
+        <v>0.022</v>
       </c>
       <c r="D43" t="s">
         <v>45</v>
@@ -1501,13 +1501,13 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B44">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C44">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="D44" t="s">
         <v>46</v>
@@ -1515,13 +1515,13 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B45">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C45">
-        <v>0</v>
+        <v>0.804</v>
       </c>
       <c r="D45" t="s">
         <v>47</v>
@@ -1529,13 +1529,13 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B46">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C46">
-        <v>0.022</v>
+        <v>1.665</v>
       </c>
       <c r="D46" t="s">
         <v>48</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B47">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C47">
-        <v>0.216</v>
+        <v>2.173</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B48">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C48">
-        <v>0.823</v>
+        <v>2.963</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B49">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C49">
-        <v>1.365</v>
+        <v>3.15</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B50">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C50">
-        <v>2.251</v>
+        <v>2.352</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B51">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C51">
-        <v>2.516</v>
+        <v>3.024</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B52">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C52">
-        <v>2.592</v>
+        <v>3.105</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B53">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C53">
-        <v>2.486</v>
+        <v>2.736</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B54">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C54">
-        <v>2.206</v>
+        <v>2.272</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B55">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C55">
-        <v>1.769</v>
+        <v>1.581</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B56">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C56">
-        <v>1.725</v>
+        <v>0.758</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B57">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C57">
-        <v>1.425</v>
+        <v>0.237</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B58">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C58">
-        <v>1.075</v>
+        <v>0.04</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B59">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C59">
-        <v>0.633</v>
+        <v>0</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,13 +1725,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B60">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C60">
-        <v>0.178</v>
+        <v>0</v>
       </c>
       <c r="D60" t="s">
         <v>62</v>
@@ -1739,13 +1739,13 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46175</v>
+        <v>46178</v>
       </c>
       <c r="B61">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C61">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="D61" t="s">
         <v>63</v>
@@ -1753,10 +1753,10 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B62">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -1767,10 +1767,10 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B63">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -1781,10 +1781,10 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B64">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -1795,10 +1795,10 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B65">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -1809,10 +1809,10 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B66">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -1823,13 +1823,13 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B67">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C67">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="D67" t="s">
         <v>69</v>
@@ -1837,13 +1837,13 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B68">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C68">
-        <v>0</v>
+        <v>0.335</v>
       </c>
       <c r="D68" t="s">
         <v>70</v>
@@ -1851,13 +1851,13 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B69">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C69">
-        <v>0</v>
+        <v>1.124</v>
       </c>
       <c r="D69" t="s">
         <v>71</v>
@@ -1865,13 +1865,13 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B70">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C70">
-        <v>0.028</v>
+        <v>2.072</v>
       </c>
       <c r="D70" t="s">
         <v>72</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B71">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C71">
-        <v>0.308</v>
+        <v>3.127</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B72">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C72">
-        <v>1.207</v>
+        <v>2.42</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B73">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C73">
-        <v>2.232</v>
+        <v>1.956</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B74">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C74">
-        <v>3.014</v>
+        <v>3.382</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B75">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C75">
-        <v>3.233</v>
+        <v>3.678</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B76">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C76">
-        <v>3.079</v>
+        <v>3.355</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B77">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C77">
-        <v>1.446</v>
+        <v>2.794</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B78">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C78">
-        <v>1.878</v>
+        <v>2.193</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B79">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C79">
-        <v>3.171</v>
+        <v>1.398</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B80">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C80">
-        <v>2.922</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B81">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C81">
-        <v>2.466</v>
+        <v>0.236</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B82">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C82">
-        <v>1.625</v>
+        <v>0.02</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B83">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C83">
-        <v>0.748</v>
+        <v>0</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,13 +2061,13 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B84">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C84">
-        <v>0.228</v>
+        <v>0</v>
       </c>
       <c r="D84" t="s">
         <v>86</v>
@@ -2075,13 +2075,13 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46176</v>
+        <v>46179</v>
       </c>
       <c r="B85">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C85">
-        <v>0.037</v>
+        <v>0</v>
       </c>
       <c r="D85" t="s">
         <v>87</v>
@@ -2089,10 +2089,10 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B86">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C86">
         <v>0</v>
@@ -2103,10 +2103,10 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B87">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C87">
         <v>0</v>
@@ -2117,10 +2117,10 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B88">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -2131,10 +2131,10 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B89">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -2145,10 +2145,10 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B90">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -2159,13 +2159,13 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B91">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C91">
-        <v>0</v>
+        <v>0.027</v>
       </c>
       <c r="D91" t="s">
         <v>93</v>
@@ -2173,13 +2173,13 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B92">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C92">
-        <v>0</v>
+        <v>0.272</v>
       </c>
       <c r="D92" t="s">
         <v>94</v>
@@ -2187,13 +2187,13 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B93">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C93">
-        <v>0</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="D93" t="s">
         <v>95</v>
@@ -2201,13 +2201,13 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B94">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C94">
-        <v>0.036</v>
+        <v>1.676</v>
       </c>
       <c r="D94" t="s">
         <v>96</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B95">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C95">
-        <v>0.334</v>
+        <v>2.087</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B96">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C96">
-        <v>1.182</v>
+        <v>2.598</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B97">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C97">
-        <v>2.172</v>
+        <v>2.897</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B98">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C98">
-        <v>3.239</v>
+        <v>2.71</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B99">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C99">
-        <v>3.294</v>
+        <v>2.75</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B100">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C100">
-        <v>1.705</v>
+        <v>2.753</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B101">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C101">
-        <v>1.624</v>
+        <v>2.714</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B102">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C102">
-        <v>1.796</v>
+        <v>2.138</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B103">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C103">
-        <v>2.776</v>
+        <v>1.359</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B104">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C104">
-        <v>2.893</v>
+        <v>0.762</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B105">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C105">
-        <v>2.31</v>
+        <v>0.236</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B106">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C106">
-        <v>1.241</v>
+        <v>0.028</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B107">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C107">
-        <v>0.746</v>
+        <v>0</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,13 +2397,13 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B108">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C108">
-        <v>0.215</v>
+        <v>0</v>
       </c>
       <c r="D108" t="s">
         <v>110</v>
@@ -2411,13 +2411,13 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46177</v>
+        <v>46180</v>
       </c>
       <c r="B109">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C109">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="D109" t="s">
         <v>111</v>
@@ -2425,10 +2425,10 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B110">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -2439,10 +2439,10 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B111">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -2453,10 +2453,10 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B112">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -2467,10 +2467,10 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B113">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -2481,10 +2481,10 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B114">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C114">
         <v>0</v>
@@ -2495,13 +2495,13 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B115">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C115">
-        <v>0</v>
+        <v>0.022</v>
       </c>
       <c r="D115" t="s">
         <v>117</v>
@@ -2509,13 +2509,13 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B116">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C116">
-        <v>0</v>
+        <v>0.211</v>
       </c>
       <c r="D116" t="s">
         <v>118</v>
@@ -2523,13 +2523,13 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B117">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C117">
-        <v>0</v>
+        <v>0.725</v>
       </c>
       <c r="D117" t="s">
         <v>119</v>
@@ -2537,13 +2537,13 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B118">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C118">
-        <v>0.028</v>
+        <v>1.267</v>
       </c>
       <c r="D118" t="s">
         <v>120</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B119">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C119">
-        <v>0.312</v>
+        <v>1.78</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B120">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C120">
-        <v>1.084</v>
+        <v>2.092</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B121">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C121">
-        <v>2.042</v>
+        <v>2.447</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B122">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C122">
-        <v>2.437</v>
+        <v>2.858</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B123">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C123">
-        <v>3.285</v>
+        <v>2.903</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B124">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C124">
-        <v>2.829</v>
+        <v>2.744</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B125">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C125">
-        <v>1.463</v>
+        <v>2.739</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B126">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C126">
-        <v>1.443</v>
+        <v>2.309</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B127">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C127">
-        <v>1.865</v>
+        <v>1.58</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B128">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C128">
-        <v>2.807</v>
+        <v>0.829</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B129">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C129">
-        <v>2.469</v>
+        <v>0.231</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B130">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C130">
-        <v>1.604</v>
+        <v>0.037</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B131">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C131">
-        <v>0.792</v>
+        <v>0</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,13 +2733,13 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B132">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C132">
-        <v>0.224</v>
+        <v>0</v>
       </c>
       <c r="D132" t="s">
         <v>134</v>
@@ -2747,13 +2747,13 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B133">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C133">
-        <v>0.037</v>
+        <v>0</v>
       </c>
       <c r="D133" t="s">
         <v>135</v>
@@ -2761,10 +2761,10 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B134">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -2775,10 +2775,10 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B135">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C135">
         <v>0</v>
@@ -2789,10 +2789,10 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B136">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C136">
         <v>0</v>
@@ -2803,10 +2803,10 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B137">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C137">
         <v>0</v>
@@ -2817,10 +2817,10 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B138">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -2831,13 +2831,13 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B139">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C139">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="D139" t="s">
         <v>141</v>
@@ -2845,13 +2845,13 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B140">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C140">
-        <v>0</v>
+        <v>0.33</v>
       </c>
       <c r="D140" t="s">
         <v>142</v>
@@ -2859,13 +2859,13 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B141">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C141">
-        <v>0</v>
+        <v>1.137</v>
       </c>
       <c r="D141" t="s">
         <v>143</v>
@@ -2873,13 +2873,13 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B142">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C142">
-        <v>0.035</v>
+        <v>2.165</v>
       </c>
       <c r="D142" t="s">
         <v>144</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B143">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C143">
-        <v>0.331</v>
+        <v>2.683</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B144">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C144">
-        <v>1.111</v>
+        <v>3.103</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B145">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C145">
-        <v>2.13</v>
+        <v>3.175</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B146">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C146">
-        <v>3.183</v>
+        <v>3.225</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B147">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C147">
-        <v>2.926</v>
+        <v>3.209</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B148">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C148">
-        <v>1.854</v>
+        <v>2.887</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B149">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C149">
-        <v>1.77</v>
+        <v>2.647</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B150">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C150">
-        <v>3.256</v>
+        <v>2.115</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B151">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C151">
-        <v>3.378</v>
+        <v>1.151</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B152">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C152">
-        <v>3.017</v>
+        <v>0.664</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B153">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C153">
-        <v>2.507</v>
+        <v>0.223</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B154">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C154">
-        <v>1.66</v>
+        <v>0.025</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B155">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C155">
-        <v>0.781</v>
+        <v>0</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,13 +3069,13 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B156">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C156">
-        <v>0.239</v>
+        <v>0</v>
       </c>
       <c r="D156" t="s">
         <v>158</v>
@@ -3083,13 +3083,13 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46179</v>
+        <v>46182</v>
       </c>
       <c r="B157">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C157">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="D157" t="s">
         <v>159</v>
@@ -3097,10 +3097,10 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B158">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -3111,10 +3111,10 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B159">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C159">
         <v>0</v>
@@ -3125,10 +3125,10 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B160">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C160">
         <v>0</v>
@@ -3139,10 +3139,10 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B161">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C161">
         <v>0</v>
@@ -3153,10 +3153,10 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B162">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C162">
         <v>0</v>
@@ -3167,13 +3167,13 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B163">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C163">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="D163" t="s">
         <v>165</v>
@@ -3181,13 +3181,13 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B164">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C164">
-        <v>0</v>
+        <v>0.343</v>
       </c>
       <c r="D164" t="s">
         <v>166</v>
@@ -3195,13 +3195,13 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B165">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C165">
-        <v>0</v>
+        <v>1.076</v>
       </c>
       <c r="D165" t="s">
         <v>167</v>
@@ -3209,13 +3209,13 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B166">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C166">
-        <v>0.035</v>
+        <v>2.063</v>
       </c>
       <c r="D166" t="s">
         <v>168</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B167">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C167">
-        <v>0.336</v>
+        <v>2.441</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B168">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C168">
-        <v>1.134</v>
+        <v>3.032</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B169">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C169">
-        <v>2.045</v>
+        <v>3.332</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46180</v>
+        <v>46183</v>
       </c>
       <c r="B170">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C170">
-        <v>2.72</v>
+        <v>3.408</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>